<commit_message>
T-0839: settle the derivation chain, raise the two spend ceilings with reasons, wire the gate
</commit_message>
<xml_diff>
--- a/chicago/reference/resident-research/T-0442/T-0442_resident_research_working.xlsx
+++ b/chicago/reference/resident-research/T-0442/T-0442_resident_research_working.xlsx
@@ -878,7 +878,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>andreas_1884_v1; chicago_democrat_1833_11_26; chicago_voter_lists_1833_1835_irad</t>
+          <t>andreas_1884_v1; chicago_democrat_1833_11_26; chicago_democrat_1833_1835; chicago_voter_lists_1833_1835_irad; fergus_chicago_directory_1839</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>andreas_1884_v1; chicago_voter_lists_1833_1835_irad</t>
+          <t>andreas_1884_v1; calumet_club_early_chicago_1879; census_1840_chicago_familysearch_images; chicago_american_1835; chicago_democrat_1833_1835; chicago_voter_lists_1833_1835_irad; fergus_chicago_directory_1843; norris_directory_1844</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>

</xml_diff>